<commit_message>
Add original templates and interface screenshots
</commit_message>
<xml_diff>
--- a/templates/border_inspection_procedures_template.xlsx
+++ b/templates/border_inspection_procedures_template.xlsx
@@ -5,11 +5,11 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PublicTemplates\0806锦耀\打印\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\UA\Desktop\0814埃莱夫塞里娅\打印\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="12255"/>
+    <workbookView windowWidth="17820" windowHeight="12255"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,15 +37,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="32">
   <si>
     <t>边检手续办理信息表</t>
   </si>
   <si>
-    <t>大船船名：中文：锦耀                英文：ASL TAIPEI</t>
-  </si>
-  <si>
-    <t>船舶公司名称（请填写完整准确名称）：上海锦江航运（集团）有限公司</t>
+    <t>大船船名：中文：埃莱夫塞里娅                英文：GSL ELEFTHERIA</t>
+  </si>
+  <si>
+    <t>船舶公司名称（请填写完整准确名称）：马士基（中国）航运有限公司青岛分公司</t>
   </si>
   <si>
     <t>海关是否需要核酸检测或登轮检查</t>
@@ -57,123 +57,28 @@
     <t>抵达时间</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>计划驶离时间</t>
   </si>
   <si>
     <t>来自港</t>
   </si>
   <si>
-    <t>越南胡志明</t>
+    <t>香港</t>
   </si>
   <si>
     <t>目的港</t>
   </si>
   <si>
-    <t>日本博多</t>
+    <t>林查班</t>
   </si>
   <si>
     <t>证件种类情况</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve">中国籍海员证：19 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Tahoma"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>本；</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Tahoma"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve">  </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>外国籍护照：   本；</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Tahoma"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve">  </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>外国籍海员证：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Tahoma"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve">   </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>本；港澳台证件：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Tahoma"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve">   </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>本（张）</t>
-    </r>
+    <t>中国籍海员证： 0 本；  外国籍护照： 19 本；  外国籍海员证： 0 本；港澳台证件： 0 本（张）</t>
   </si>
   <si>
     <t>有无女性船员</t>
@@ -185,6 +90,9 @@
     <t>女性船员数量</t>
   </si>
   <si>
+    <t>0</t>
+  </si>
+  <si>
     <t>本港有无船员变动</t>
   </si>
   <si>
@@ -203,13 +111,13 @@
     <t>国内航次情况</t>
   </si>
   <si>
-    <t>越南胡志明-南沙-日本博多；</t>
+    <t>香港-南沙-林查班；</t>
   </si>
   <si>
     <t>停靠码头泊位</t>
   </si>
   <si>
-    <t>南沙一期     号泊位</t>
+    <t>南沙二期六号泊位</t>
   </si>
   <si>
     <t>是否携带枪支弹药</t>
@@ -1609,122 +1517,132 @@
       <c r="A5" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="15"/>
+      <c r="B5" s="15" t="s">
+        <v>6</v>
+      </c>
       <c r="C5" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="15"/>
     </row>
     <row r="6" ht="27" customHeight="1" spans="1:4">
       <c r="A6" s="14" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" ht="27" customHeight="1" spans="1:4">
       <c r="A7" s="14" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C7" s="17"/>
       <c r="D7" s="17"/>
     </row>
     <row r="8" ht="27" customHeight="1" spans="1:4">
       <c r="A8" s="14" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="D8" s="15"/>
+        <v>16</v>
+      </c>
+      <c r="D8" s="15" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="9" ht="27" customHeight="1" spans="1:4">
       <c r="A9" s="14" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="D9" s="18"/>
+        <v>19</v>
+      </c>
+      <c r="D9" s="18" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="10" ht="27" customHeight="1" spans="1:4">
       <c r="A10" s="14" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="D10" s="18"/>
+        <v>19</v>
+      </c>
+      <c r="D10" s="18" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="11" ht="37.5" spans="1:4">
       <c r="A11" s="19" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B11" s="15"/>
       <c r="C11" s="14" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D11" s="15"/>
     </row>
     <row r="12" ht="67.05" customHeight="1" spans="1:4">
       <c r="A12" s="19" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B12" s="20" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C12" s="21"/>
       <c r="D12" s="22"/>
     </row>
     <row r="13" ht="27" customHeight="1" spans="1:4">
       <c r="A13" s="19" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C13" s="24"/>
       <c r="D13" s="25"/>
     </row>
     <row r="14" ht="27" customHeight="1" spans="1:4">
       <c r="A14" s="14" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15" ht="21" customHeight="1" spans="1:4">
       <c r="A15" s="26" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B15" s="27" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C15" s="27"/>
       <c r="D15" s="28"/>

</xml_diff>

<commit_message>
Fix form exports and preserve customs logo
</commit_message>
<xml_diff>
--- a/templates/border_inspection_procedures_template.xlsx
+++ b/templates/border_inspection_procedures_template.xlsx
@@ -5,11 +5,11 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\UA\Desktop\0814埃莱夫塞里娅\打印\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PublicTemplates\0806锦耀\打印\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="17820" windowHeight="12255"/>
+    <workbookView windowWidth="27945" windowHeight="12255"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,15 +37,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="30">
   <si>
     <t>边检手续办理信息表</t>
   </si>
   <si>
-    <t>大船船名：中文：埃莱夫塞里娅                英文：GSL ELEFTHERIA</t>
-  </si>
-  <si>
-    <t>船舶公司名称（请填写完整准确名称）：马士基（中国）航运有限公司青岛分公司</t>
+    <t>大船船名：中文：锦耀                英文：ASL TAIPEI</t>
+  </si>
+  <si>
+    <t>船舶公司名称（请填写完整准确名称）：上海锦江航运（集团）有限公司</t>
   </si>
   <si>
     <t>海关是否需要核酸检测或登轮检查</t>
@@ -57,28 +57,123 @@
     <t>抵达时间</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>计划驶离时间</t>
   </si>
   <si>
     <t>来自港</t>
   </si>
   <si>
-    <t>香港</t>
+    <t>越南胡志明</t>
   </si>
   <si>
     <t>目的港</t>
   </si>
   <si>
-    <t>林查班</t>
+    <t>日本博多</t>
   </si>
   <si>
     <t>证件种类情况</t>
   </si>
   <si>
-    <t>中国籍海员证： 0 本；  外国籍护照： 19 本；  外国籍海员证： 0 本；港澳台证件： 0 本（张）</t>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">中国籍海员证：19 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>本；</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>外国籍护照：   本；</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>外国籍海员证：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">   </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>本；港澳台证件：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">   </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>本（张）</t>
+    </r>
   </si>
   <si>
     <t>有无女性船员</t>
@@ -90,9 +185,6 @@
     <t>女性船员数量</t>
   </si>
   <si>
-    <t>0</t>
-  </si>
-  <si>
     <t>本港有无船员变动</t>
   </si>
   <si>
@@ -111,13 +203,13 @@
     <t>国内航次情况</t>
   </si>
   <si>
-    <t>香港-南沙-林查班；</t>
+    <t>越南胡志明-南沙-日本博多；</t>
   </si>
   <si>
     <t>停靠码头泊位</t>
   </si>
   <si>
-    <t>南沙二期六号泊位</t>
+    <t>南沙一期     号泊位</t>
   </si>
   <si>
     <t>是否携带枪支弹药</t>
@@ -1517,132 +1609,122 @@
       <c r="A5" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="15"/>
+      <c r="C5" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="15" t="s">
-        <v>6</v>
-      </c>
+      <c r="D5" s="15"/>
     </row>
     <row r="6" ht="27" customHeight="1" spans="1:4">
       <c r="A6" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="16" t="s">
+      <c r="C6" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="D6" s="16" t="s">
         <v>10</v>
-      </c>
-      <c r="D6" s="16" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="7" ht="27" customHeight="1" spans="1:4">
       <c r="A7" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="14" t="s">
         <v>12</v>
-      </c>
-      <c r="B7" s="14" t="s">
-        <v>13</v>
       </c>
       <c r="C7" s="17"/>
       <c r="D7" s="17"/>
     </row>
     <row r="8" ht="27" customHeight="1" spans="1:4">
       <c r="A8" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="C8" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="D8" s="15" t="s">
-        <v>17</v>
-      </c>
+      <c r="D8" s="15"/>
     </row>
     <row r="9" ht="27" customHeight="1" spans="1:4">
       <c r="A9" s="14" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="D9" s="18" t="s">
-        <v>6</v>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="D9" s="18"/>
     </row>
     <row r="10" ht="27" customHeight="1" spans="1:4">
       <c r="A10" s="14" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="D10" s="18" t="s">
-        <v>6</v>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="D10" s="18"/>
     </row>
     <row r="11" ht="37.5" spans="1:4">
       <c r="A11" s="19" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B11" s="15"/>
       <c r="C11" s="14" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D11" s="15"/>
     </row>
     <row r="12" ht="67.05" customHeight="1" spans="1:4">
       <c r="A12" s="19" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B12" s="20" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C12" s="21"/>
       <c r="D12" s="22"/>
     </row>
     <row r="13" ht="27" customHeight="1" spans="1:4">
       <c r="A13" s="19" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C13" s="24"/>
       <c r="D13" s="25"/>
     </row>
     <row r="14" ht="27" customHeight="1" spans="1:4">
       <c r="A14" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="B14" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="C14" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="18" t="s">
-        <v>28</v>
-      </c>
-      <c r="C14" s="14" t="s">
-        <v>29</v>
-      </c>
       <c r="D14" s="18" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15" ht="21" customHeight="1" spans="1:4">
       <c r="A15" s="26" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B15" s="27" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C15" s="27"/>
       <c r="D15" s="28"/>

</xml_diff>